<commit_message>
checkup: run only when market is closed, self-computed RVOL with consistency check, Drive replace flow
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0145VbtPApM8bCdkcpH6K5ee
</commit_message>
<xml_diff>
--- a/checkup_data/Summary of 2026-10-22.xlsx
+++ b/checkup_data/Summary of 2026-10-22.xlsx
@@ -704,7 +704,7 @@
         <v>84.621</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>0.769</v>
+        <v>0.785221762798584</v>
       </c>
       <c r="J2" s="6" t="n">
         <v>3.3775</v>
@@ -781,11 +781,11 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
@@ -803,95 +803,95 @@
         </is>
       </c>
       <c r="F3" s="6" t="n">
+        <v>149.88</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>1.065407956844222</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>128.837</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>0.9154647073884273</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>3.9256</v>
+      </c>
+      <c r="K3" s="8" t="n">
+        <v>2.619161996263678</v>
+      </c>
+      <c r="L3" s="8" t="n">
+        <v>15.544</v>
+      </c>
+      <c r="M3" s="8" t="n">
+        <v>25.926</v>
+      </c>
+      <c r="N3" s="8" t="n">
+        <v>18.861</v>
+      </c>
+      <c r="O3" s="8" t="n">
+        <v>57.88</v>
+      </c>
+      <c r="P3" s="6" t="n">
+        <v>145.745</v>
+      </c>
+      <c r="Q3" s="6" t="n">
+        <v>143.237</v>
+      </c>
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>ירוק</t>
+        </is>
+      </c>
+      <c r="S3" s="9" t="n">
+        <v>0.9584775086505173</v>
+      </c>
+      <c r="T3" s="10" t="inlineStr">
+        <is>
+          <t>נר גוף מלא ירוק</t>
+        </is>
+      </c>
+      <c r="U3" s="6" t="n">
+        <v>151.813</v>
+      </c>
+      <c r="V3" s="11" t="inlineStr">
+        <is>
+          <t>R1 M</t>
+        </is>
+      </c>
+      <c r="W3" s="8" t="n">
+        <v>0.4924088037497434</v>
+      </c>
+      <c r="X3" s="6" t="n">
         <v>153.57</v>
       </c>
-      <c r="G3" s="7" t="n">
-        <v>-1.878474218899751</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>137.615</v>
-      </c>
-      <c r="I3" s="6" t="n">
-        <v>1.017</v>
-      </c>
-      <c r="J3" s="6" t="n">
-        <v>3.9414</v>
-      </c>
-      <c r="K3" s="8" t="n">
-        <v>2.566516897831608</v>
-      </c>
-      <c r="L3" s="8" t="n">
-        <v>22.874</v>
-      </c>
-      <c r="M3" s="8" t="n">
-        <v>26.96</v>
-      </c>
-      <c r="N3" s="8" t="n">
-        <v>20.413</v>
-      </c>
-      <c r="O3" s="8" t="n">
-        <v>55.74</v>
-      </c>
-      <c r="P3" s="6" t="n">
-        <v>151.201</v>
-      </c>
-      <c r="Q3" s="6" t="n">
-        <v>147.194</v>
-      </c>
-      <c r="R3" s="5" t="inlineStr">
-        <is>
-          <t>אדום</t>
-        </is>
-      </c>
-      <c r="S3" s="9" t="n">
-        <v>0.3126684636118606</v>
-      </c>
-      <c r="T3" s="10" t="inlineStr">
-        <is>
-          <t>נר אדום</t>
-        </is>
-      </c>
-      <c r="U3" s="6" t="n">
-        <v>154.6533333333333</v>
-      </c>
-      <c r="V3" s="11" t="inlineStr">
-        <is>
-          <t>נמוך קודם+R1 M+גבוה אחרון</t>
-        </is>
-      </c>
-      <c r="W3" s="8" t="n">
-        <v>0.2748600328140617</v>
-      </c>
-      <c r="X3" s="6" t="n">
-        <v>157.48</v>
-      </c>
       <c r="Y3" s="6" t="n">
-        <v>151.4555</v>
+        <v>149.68</v>
       </c>
       <c r="Z3" s="11" t="inlineStr">
         <is>
-          <t>EMA20+נמוך אחרון</t>
+          <t>גבוה קודם+גבוה אחרון</t>
         </is>
       </c>
       <c r="AA3" s="8" t="n">
-        <v>0.5364844978941474</v>
+        <v>0.05094762584063293</v>
       </c>
       <c r="AB3" s="6" t="n">
-        <v>148.73</v>
+        <v>146.5105</v>
       </c>
       <c r="AC3" s="12" t="n">
-        <v>6231242</v>
+        <v>9838589</v>
       </c>
       <c r="AD3" s="10" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
@@ -909,84 +909,84 @@
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>149.88</v>
+        <v>153.57</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>1.065407956844222</v>
+        <v>-1.878474218899751</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>128.837</v>
+        <v>137.615</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.9982730569603941</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>3.9256</v>
+        <v>3.9414</v>
       </c>
       <c r="K4" s="8" t="n">
-        <v>2.619161996263678</v>
+        <v>2.566516897831608</v>
       </c>
       <c r="L4" s="8" t="n">
-        <v>15.544</v>
+        <v>22.874</v>
       </c>
       <c r="M4" s="8" t="n">
-        <v>25.926</v>
+        <v>26.96</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>18.861</v>
+        <v>20.413</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>57.88</v>
+        <v>55.74</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>145.745</v>
+        <v>151.201</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>143.237</v>
-      </c>
-      <c r="R4" s="4" t="inlineStr">
-        <is>
-          <t>ירוק</t>
+        <v>147.194</v>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>אדום</t>
         </is>
       </c>
       <c r="S4" s="9" t="n">
-        <v>0.9584775086505173</v>
+        <v>0.3126684636118606</v>
       </c>
       <c r="T4" s="10" t="inlineStr">
         <is>
-          <t>נר גוף מלא ירוק</t>
+          <t>נר אדום</t>
         </is>
       </c>
       <c r="U4" s="6" t="n">
-        <v>151.813</v>
+        <v>154.6533333333333</v>
       </c>
       <c r="V4" s="11" t="inlineStr">
         <is>
-          <t>R1 M</t>
+          <t>נמוך קודם+R1 M+גבוה אחרון</t>
         </is>
       </c>
       <c r="W4" s="8" t="n">
-        <v>0.4924088037497434</v>
+        <v>0.2748600328140617</v>
       </c>
       <c r="X4" s="6" t="n">
-        <v>153.57</v>
+        <v>157.48</v>
       </c>
       <c r="Y4" s="6" t="n">
-        <v>149.68</v>
+        <v>151.4555</v>
       </c>
       <c r="Z4" s="11" t="inlineStr">
         <is>
-          <t>גבוה קודם+גבוה אחרון</t>
+          <t>EMA20+נמוך אחרון</t>
         </is>
       </c>
       <c r="AA4" s="8" t="n">
-        <v>0.05094762584063293</v>
+        <v>0.5364844978941474</v>
       </c>
       <c r="AB4" s="6" t="n">
-        <v>146.5105</v>
+        <v>148.73</v>
       </c>
       <c r="AC4" s="12" t="n">
-        <v>9838589</v>
+        <v>6231242</v>
       </c>
       <c r="AD4" s="10" t="inlineStr"/>
     </row>
@@ -1024,7 +1024,7 @@
         <v>15.011</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>1.407</v>
+        <v>1.419540790535567</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>1.1519</v>
@@ -1130,7 +1130,7 @@
         <v>32.803</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>1.477</v>
+        <v>1.409305291538969</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>1.9007</v>
@@ -1205,7 +1205,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>OMDA</t>
+          <t>TVTX</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
@@ -1216,9 +1216,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>❌</t>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1227,84 +1227,84 @@
         </is>
       </c>
       <c r="F7" s="6" t="n">
-        <v>19.66</v>
+        <v>52.58</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>1.654601861427096</v>
+        <v>0.5353728489483789</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>18.8</v>
+        <v>51.373</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>1.039</v>
+        <v>1.249768718765484</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>1.0868</v>
+        <v>2.3741</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>5.527975584944049</v>
+        <v>4.5152149106124</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>17.331</v>
+        <v>29.875</v>
       </c>
       <c r="M7" s="8" t="n">
-        <v>23.185</v>
+        <v>23.392</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>27.381</v>
+        <v>25.628</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>47.7</v>
+        <v>38.86</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>19.775</v>
+        <v>54.775</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>20.524</v>
-      </c>
-      <c r="R7" s="4" t="inlineStr">
-        <is>
-          <t>ירוק</t>
+        <v>57.529</v>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>אדום</t>
         </is>
       </c>
       <c r="S7" s="9" t="n">
-        <v>0.4943820224719073</v>
+        <v>0.1287553648068689</v>
       </c>
       <c r="T7" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>פטיש הפוך (Inverted Hammer)</t>
         </is>
       </c>
       <c r="U7" s="6" t="n">
-        <v>19.785</v>
+        <v>54.94266666666667</v>
       </c>
       <c r="V7" s="11" t="inlineStr">
         <is>
-          <t>EMA20+גבוה אחרון</t>
+          <t>EMA20+גבוה אחרון+S1 M</t>
         </is>
       </c>
       <c r="W7" s="8" t="n">
-        <v>0.1150165623849834</v>
+        <v>0.995184139954791</v>
       </c>
       <c r="X7" s="6" t="n">
-        <v>20.524</v>
+        <v>57.529</v>
       </c>
       <c r="Y7" s="6" t="n">
-        <v>19.355</v>
+        <v>51.567</v>
       </c>
       <c r="Z7" s="11" t="inlineStr">
         <is>
-          <t>נמוך אחרון+גבוה קודם</t>
+          <t>S2 M</t>
         </is>
       </c>
       <c r="AA7" s="8" t="n">
-        <v>0.2806404122193593</v>
+        <v>0.4266880080872744</v>
       </c>
       <c r="AB7" s="6" t="n">
-        <v>18.0915</v>
+        <v>50.4</v>
       </c>
       <c r="AC7" s="12" t="n">
-        <v>1254460</v>
+        <v>1731658</v>
       </c>
       <c r="AD7" s="10" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BEN</t>
+          <t>OMDA</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
@@ -1337,40 +1337,40 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>31.68</v>
+        <v>19.66</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>1.40845070422535</v>
+        <v>1.654601861427096</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>31.304</v>
+        <v>18.8</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>0.628</v>
+        <v>1.03518406326228</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>0.8166</v>
+        <v>1.0868</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>2.577651515151515</v>
+        <v>5.527975584944049</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>29.128</v>
+        <v>17.331</v>
       </c>
       <c r="M8" s="8" t="n">
-        <v>17.623</v>
+        <v>23.185</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>24.645</v>
+        <v>27.381</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>45.28</v>
+        <v>47.7</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>31.915</v>
+        <v>19.775</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>32.563</v>
+        <v>20.524</v>
       </c>
       <c r="R8" s="4" t="inlineStr">
         <is>
@@ -1378,43 +1378,43 @@
         </is>
       </c>
       <c r="S8" s="9" t="n">
-        <v>0.1799999999999997</v>
+        <v>0.4943820224719073</v>
       </c>
       <c r="T8" s="10" t="inlineStr">
         <is>
-          <t>פטיש (Hammer)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U8" s="6" t="n">
-        <v>31.76166666666667</v>
+        <v>19.785</v>
       </c>
       <c r="V8" s="11" t="inlineStr">
         <is>
-          <t>גבוה קודם+גבוה אחרון+EMA20</t>
+          <t>EMA20+גבוה אחרון</t>
         </is>
       </c>
       <c r="W8" s="8" t="n">
-        <v>0.1000081639317499</v>
+        <v>0.1150165623849834</v>
       </c>
       <c r="X8" s="6" t="n">
-        <v>32.563</v>
+        <v>20.524</v>
       </c>
       <c r="Y8" s="6" t="n">
-        <v>31.25</v>
+        <v>19.355</v>
       </c>
       <c r="Z8" s="11" t="inlineStr">
         <is>
-          <t>נמוך אחרון</t>
+          <t>נמוך אחרון+גבוה קודם</t>
         </is>
       </c>
       <c r="AA8" s="8" t="n">
-        <v>0.5265735978447217</v>
+        <v>0.2806404122193593</v>
       </c>
       <c r="AB8" s="6" t="n">
-        <v>31.033</v>
+        <v>18.0915</v>
       </c>
       <c r="AC8" s="12" t="n">
-        <v>3903043</v>
+        <v>1254460</v>
       </c>
       <c r="AD8" s="10" t="inlineStr">
         <is>
@@ -1425,11 +1425,11 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TARS</t>
+          <t>BEN</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
@@ -1441,101 +1441,105 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>מעורבת</t>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>יורדת ▼</t>
         </is>
       </c>
       <c r="F9" s="6" t="n">
-        <v>70.5</v>
+        <v>31.68</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>-0.7461635928480925</v>
+        <v>1.40845070422535</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>67.252</v>
+        <v>31.304</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>0.803</v>
+        <v>0.6578526037248372</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3.187</v>
+        <v>0.8166</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>4.520567375886524</v>
+        <v>2.577651515151515</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>15.554</v>
+        <v>29.128</v>
       </c>
       <c r="M9" s="8" t="n">
-        <v>17.585</v>
+        <v>17.623</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>19.997</v>
+        <v>24.645</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>43.33</v>
+        <v>45.28</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>72.786</v>
+        <v>31.915</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>72.729</v>
-      </c>
-      <c r="R9" s="5" t="inlineStr">
-        <is>
-          <t>אדום</t>
+        <v>32.563</v>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
+        <is>
+          <t>ירוק</t>
         </is>
       </c>
       <c r="S9" s="9" t="n">
-        <v>0.1340996168582354</v>
+        <v>0.1799999999999997</v>
       </c>
       <c r="T9" s="10" t="inlineStr">
         <is>
-          <t>פטיש הפוך (Inverted Hammer)</t>
+          <t>פטיש (Hammer)</t>
         </is>
       </c>
       <c r="U9" s="6" t="n">
-        <v>72.69624999999999</v>
+        <v>31.76166666666667</v>
       </c>
       <c r="V9" s="11" t="inlineStr">
         <is>
-          <t>גבוה קודם+EMA50+EMA20+גבוה אחרון</t>
+          <t>גבוה קודם+גבוה אחרון+EMA20</t>
         </is>
       </c>
       <c r="W9" s="8" t="n">
-        <v>0.6891277063068693</v>
+        <v>0.1000081639317499</v>
       </c>
       <c r="X9" s="6" t="n">
-        <v>79.09999999999999</v>
+        <v>32.563</v>
       </c>
       <c r="Y9" s="6" t="n">
-        <v>67.93000000000001</v>
+        <v>31.25</v>
       </c>
       <c r="Z9" s="11" t="inlineStr">
         <is>
-          <t>נמוך קודם+שפל חודש</t>
+          <t>נמוך אחרון</t>
         </is>
       </c>
       <c r="AA9" s="8" t="n">
-        <v>0.8064010040790691</v>
+        <v>0.5265735978447217</v>
       </c>
       <c r="AB9" s="6" t="n">
-        <v>63.203</v>
+        <v>31.033</v>
       </c>
       <c r="AC9" s="12" t="n">
-        <v>1218388</v>
-      </c>
-      <c r="AD9" s="10" t="inlineStr"/>
+        <v>3903043</v>
+      </c>
+      <c r="AD9" s="10" t="inlineStr">
+        <is>
+          <t>מגמת ירידה — לונג נגד המגמה</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BNY</t>
+          <t>TARS</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
@@ -1553,91 +1557,91 @@
         </is>
       </c>
       <c r="F10" s="6" t="n">
-        <v>145.85</v>
+        <v>70.5</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>1.109185441941074</v>
+        <v>-0.7461635928480925</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>144.825</v>
+        <v>67.252</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.7763602399235712</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>3.2132</v>
+        <v>3.187</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>2.203085361672952</v>
+        <v>4.520567375886524</v>
       </c>
       <c r="L10" s="8" t="n">
-        <v>31.076</v>
+        <v>15.554</v>
       </c>
       <c r="M10" s="8" t="n">
-        <v>24.788</v>
+        <v>17.585</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>27.116</v>
+        <v>19.997</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>47.7</v>
+        <v>43.33</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>145.3</v>
+        <v>72.786</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>149.493</v>
-      </c>
-      <c r="R10" s="4" t="inlineStr">
-        <is>
-          <t>ירוק</t>
+        <v>72.729</v>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>אדום</t>
         </is>
       </c>
       <c r="S10" s="9" t="n">
-        <v>0.04113110539844955</v>
+        <v>0.1340996168582354</v>
       </c>
       <c r="T10" s="10" t="inlineStr">
         <is>
-          <t>דוג'י</t>
+          <t>פטיש הפוך (Inverted Hammer)</t>
         </is>
       </c>
       <c r="U10" s="6" t="n">
-        <v>146.855</v>
+        <v>72.69624999999999</v>
       </c>
       <c r="V10" s="11" t="inlineStr">
         <is>
-          <t>גבוה אחרון</t>
+          <t>גבוה קודם+EMA50+EMA20+גבוה אחרון</t>
         </is>
       </c>
       <c r="W10" s="8" t="n">
-        <v>0.3127723142039074</v>
+        <v>0.6891277063068693</v>
       </c>
       <c r="X10" s="6" t="n">
-        <v>149.493</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="Y10" s="6" t="n">
-        <v>145.175</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="Z10" s="11" t="inlineStr">
         <is>
-          <t>נמוך אחרון+EMA20+גבוה קודם</t>
+          <t>נמוך קודם+שפל חודש</t>
         </is>
       </c>
       <c r="AA10" s="8" t="n">
-        <v>0.2100709573011364</v>
+        <v>0.8064010040790691</v>
       </c>
       <c r="AB10" s="6" t="n">
-        <v>142.05</v>
+        <v>63.203</v>
       </c>
       <c r="AC10" s="12" t="n">
-        <v>4508722</v>
+        <v>1218388</v>
       </c>
       <c r="AD10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>VOYA</t>
+          <t>BNY</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
@@ -1659,48 +1663,48 @@
         </is>
       </c>
       <c r="F11" s="6" t="n">
-        <v>96.34</v>
+        <v>145.85</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.7635184604120937</v>
+        <v>1.109185441941074</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>89.721</v>
+        <v>144.825</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>0.735</v>
+        <v>0.6750101248202928</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>2.2498</v>
+        <v>3.2132</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>2.335270915507577</v>
+        <v>2.203085361672952</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>25.544</v>
+        <v>31.076</v>
       </c>
       <c r="M11" s="8" t="n">
-        <v>20.137</v>
+        <v>24.788</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>23.194</v>
+        <v>27.116</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>48.52</v>
+        <v>47.7</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>96.2</v>
+        <v>145.3</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>97.15600000000001</v>
-      </c>
-      <c r="R11" s="11" t="inlineStr">
-        <is>
-          <t>ניטרלי</t>
+        <v>149.493</v>
+      </c>
+      <c r="R11" s="4" t="inlineStr">
+        <is>
+          <t>ירוק</t>
         </is>
       </c>
       <c r="S11" s="9" t="n">
-        <v>0</v>
+        <v>0.04113110539844955</v>
       </c>
       <c r="T11" s="10" t="inlineStr">
         <is>
@@ -1708,46 +1712,46 @@
         </is>
       </c>
       <c r="U11" s="6" t="n">
-        <v>96.58920000000001</v>
+        <v>146.855</v>
       </c>
       <c r="V11" s="11" t="inlineStr">
         <is>
-          <t>נמוך אחרון+EMA20+גבוה קודם+גבוה אחרון+EMA50</t>
+          <t>גבוה אחרון</t>
         </is>
       </c>
       <c r="W11" s="8" t="n">
-        <v>0.1107654013690114</v>
+        <v>0.3127723142039074</v>
       </c>
       <c r="X11" s="6" t="n">
-        <v>97.982</v>
+        <v>149.493</v>
       </c>
       <c r="Y11" s="6" t="n">
-        <v>93.73</v>
+        <v>145.175</v>
       </c>
       <c r="Z11" s="11" t="inlineStr">
         <is>
-          <t>נמוך קודם</t>
+          <t>נמוך אחרון+EMA20+גבוה קודם</t>
         </is>
       </c>
       <c r="AA11" s="8" t="n">
-        <v>1.160103120277358</v>
+        <v>0.2100709573011364</v>
       </c>
       <c r="AB11" s="6" t="n">
-        <v>91.84999999999999</v>
+        <v>142.05</v>
       </c>
       <c r="AC11" s="12" t="n">
-        <v>916600</v>
+        <v>4508722</v>
       </c>
       <c r="AD11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HELP</t>
+          <t>VOYA</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
@@ -1765,95 +1769,95 @@
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>10.78</v>
+        <v>96.34</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>-1.462522851919568</v>
+        <v>0.7635184604120937</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>7.899</v>
+        <v>89.721</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>0.571</v>
+        <v>0.8223707178703906</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>0.8973</v>
+        <v>2.2498</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>8.323747680890538</v>
+        <v>2.335270915507577</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>17.477</v>
+        <v>25.544</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>24.093</v>
+        <v>20.137</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>19.69</v>
+        <v>23.194</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>44.17</v>
+        <v>48.52</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>11.289</v>
+        <v>96.2</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>11.189</v>
-      </c>
-      <c r="R12" s="5" t="inlineStr">
-        <is>
-          <t>אדום</t>
+        <v>97.15600000000001</v>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>ניטרלי</t>
         </is>
       </c>
       <c r="S12" s="9" t="n">
-        <v>0.3516869985712717</v>
+        <v>0</v>
       </c>
       <c r="T12" s="10" t="inlineStr">
         <is>
-          <t>נר אדום</t>
+          <t>דוג'י</t>
         </is>
       </c>
       <c r="U12" s="6" t="n">
-        <v>11.239</v>
+        <v>96.58920000000001</v>
       </c>
       <c r="V12" s="11" t="inlineStr">
         <is>
-          <t>EMA50+EMA20</t>
+          <t>נמוך אחרון+EMA20+גבוה קודם+גבוה אחרון+EMA50</t>
         </is>
       </c>
       <c r="W12" s="8" t="n">
-        <v>0.5115346038114359</v>
+        <v>0.1107654013690114</v>
       </c>
       <c r="X12" s="6" t="n">
-        <v>11.6999</v>
+        <v>97.982</v>
       </c>
       <c r="Y12" s="6" t="n">
-        <v>10.719</v>
+        <v>93.73</v>
       </c>
       <c r="Z12" s="11" t="inlineStr">
         <is>
-          <t>נמוך קודם+S1 M+נמוך אחרון</t>
+          <t>נמוך קודם</t>
         </is>
       </c>
       <c r="AA12" s="8" t="n">
-        <v>0.06798172294661757</v>
+        <v>1.160103120277358</v>
       </c>
       <c r="AB12" s="6" t="n">
-        <v>9.970000000000001</v>
+        <v>91.84999999999999</v>
       </c>
       <c r="AC12" s="12" t="n">
-        <v>1647392</v>
+        <v>916600</v>
       </c>
       <c r="AD12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TVTX</t>
+          <t>HELP</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
@@ -1865,46 +1869,46 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>יורדת ▼</t>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>מעורבת</t>
         </is>
       </c>
       <c r="F13" s="6" t="n">
-        <v>52.58</v>
+        <v>10.78</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>0.5353728489483789</v>
+        <v>-1.462522851919568</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>51.373</v>
+        <v>7.899</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>1.165</v>
+        <v>0.5671036401779297</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>2.3741</v>
+        <v>0.8973</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>4.5152149106124</v>
+        <v>8.323747680890538</v>
       </c>
       <c r="L13" s="8" t="n">
-        <v>29.875</v>
+        <v>17.477</v>
       </c>
       <c r="M13" s="8" t="n">
-        <v>23.392</v>
+        <v>24.093</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>25.628</v>
+        <v>19.69</v>
       </c>
       <c r="O13" s="8" t="n">
-        <v>38.86</v>
+        <v>44.17</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>54.775</v>
+        <v>11.289</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>57.529</v>
+        <v>11.189</v>
       </c>
       <c r="R13" s="5" t="inlineStr">
         <is>
@@ -1912,49 +1916,45 @@
         </is>
       </c>
       <c r="S13" s="9" t="n">
-        <v>0.1287553648068689</v>
+        <v>0.3516869985712717</v>
       </c>
       <c r="T13" s="10" t="inlineStr">
         <is>
-          <t>פטיש הפוך (Inverted Hammer)</t>
+          <t>נר אדום</t>
         </is>
       </c>
       <c r="U13" s="6" t="n">
-        <v>54.94266666666667</v>
+        <v>11.239</v>
       </c>
       <c r="V13" s="11" t="inlineStr">
         <is>
-          <t>EMA20+גבוה אחרון+S1 M</t>
+          <t>EMA50+EMA20</t>
         </is>
       </c>
       <c r="W13" s="8" t="n">
-        <v>0.995184139954791</v>
+        <v>0.5115346038114359</v>
       </c>
       <c r="X13" s="6" t="n">
-        <v>57.529</v>
+        <v>11.6999</v>
       </c>
       <c r="Y13" s="6" t="n">
-        <v>51.567</v>
+        <v>10.719</v>
       </c>
       <c r="Z13" s="11" t="inlineStr">
         <is>
-          <t>S2 M</t>
+          <t>נמוך קודם+S1 M+נמוך אחרון</t>
         </is>
       </c>
       <c r="AA13" s="8" t="n">
-        <v>0.4266880080872744</v>
+        <v>0.06798172294661757</v>
       </c>
       <c r="AB13" s="6" t="n">
-        <v>50.4</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="AC13" s="12" t="n">
-        <v>1731658</v>
-      </c>
-      <c r="AD13" s="10" t="inlineStr">
-        <is>
-          <t>מגמת ירידה — לונג נגד המגמה</t>
-        </is>
-      </c>
+        <v>1647392</v>
+      </c>
+      <c r="AD13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1990,7 +1990,7 @@
         <v>86.051</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>1.116</v>
+        <v>1.090664487186713</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>2.9454</v>
@@ -2100,7 +2100,7 @@
         <v>11.347</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>0.665</v>
+        <v>0.6590386399064622</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>0.6559</v>
@@ -2210,7 +2210,7 @@
         <v>106.426</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>0.76</v>
+        <v>0.7889101345517474</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>2.1628</v>
@@ -2320,7 +2320,7 @@
         <v>50.643</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1.164</v>
+        <v>1.163882450943902</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>2.4044</v>
@@ -2430,7 +2430,7 @@
         <v>18.547</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>0.771</v>
+        <v>0.8193741934323999</v>
       </c>
       <c r="J18" s="6" t="n">
         <v>0.7706</v>
@@ -2540,7 +2540,7 @@
         <v>171.088</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>1.607</v>
+        <v>1.490796217220778</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>3.8172</v>
@@ -2650,7 +2650,7 @@
         <v>16.1</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.859</v>
+        <v>0.8799703630526056</v>
       </c>
       <c r="J20" s="6" t="n">
         <v>0.3006</v>
@@ -2760,7 +2760,7 @@
         <v>93.322</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.652</v>
+        <v>0.6659317624933356</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>2.4931</v>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>ווליום היום האחרון חלקי ממוצע 10 ימים. 1.2 ומעלה = ✅</t>
+          <t>ווליום יום המסחר האחרון שנסגר חלקי ממוצע 10 ימים. 1.2 ומעלה = ✅. בלי פרה/אפטר-מרקט</t>
         </is>
       </c>
     </row>

</xml_diff>